<commit_message>
Add initial AI run data to ai_runs.jsonl
</commit_message>
<xml_diff>
--- a/outputs/schedule_copper_cloves.xlsx
+++ b/outputs/schedule_copper_cloves.xlsx
@@ -509,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -588,8 +588,8 @@
         <is>
           <t>Copper + Cloves Mat 57
 Shruti Kulkarni
-12% pred | 12% hist
-[PROTECT_EXACT]</t>
+12% pred | 0% hist
+[]</t>
         </is>
       </c>
       <c r="C3" s="6" t="n"/>
@@ -613,152 +613,131 @@
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
-17% pred | 17% hist
-[PROTECT_EXACT]</t>
+17% pred | 0% hist
+[]</t>
         </is>
       </c>
       <c r="G4" s="6" t="n"/>
       <c r="H4" s="6" t="n"/>
     </row>
     <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+18% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
 Pushyank Nahar
 20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Pushyank Nahar
-46% pred | 46% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="n"/>
-    </row>
-    <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>09:30</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Pushyank Nahar
-21% pred | 21% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
+[]</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n"/>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+46% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="H6" s="6" t="n"/>
     </row>
     <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>11:30</t>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>17:15</t>
         </is>
       </c>
       <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+22% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Shruti Kulkarni
+27% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="6" t="n"/>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
+      <c r="H7" s="6" t="n"/>
+    </row>
+    <row r="8" ht="52" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
 Siddhartha Kusuma
-20% pred | 20% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>17:15</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-20% pred | 20% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Shruti Kulkarni
-28% pred | 28% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="n"/>
+17% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G8" s="6" t="n"/>
       <c r="H8" s="6" t="n"/>
     </row>
     <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>18:15</t>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>19:45</t>
         </is>
       </c>
       <c r="B9" s="6" t="n"/>
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-17% pred | 17% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
+Kajol Kanchan
+15% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="n"/>
       <c r="H9" s="6" t="n"/>
-    </row>
-    <row r="10" ht="52" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>19:45</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-15% pred | 15% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -774,7 +753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -853,8 +832,8 @@
         <is>
           <t>Copper + Cloves Mat 57
 Shruti Kulkarni
-12% pred | 12% hist
-[PROTECT_EXACT]</t>
+12% pred | 0% hist
+[]</t>
         </is>
       </c>
       <c r="C3" s="6" t="n"/>
@@ -878,152 +857,131 @@
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
-17% pred | 17% hist
-[PROTECT_EXACT]</t>
+17% pred | 0% hist
+[]</t>
         </is>
       </c>
       <c r="G4" s="6" t="n"/>
       <c r="H4" s="6" t="n"/>
     </row>
     <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+18% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
 Pushyank Nahar
 20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Pushyank Nahar
-46% pred | 46% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="n"/>
-    </row>
-    <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>09:30</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Pushyank Nahar
-21% pred | 21% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
+[]</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n"/>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+46% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="H6" s="6" t="n"/>
     </row>
     <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>11:30</t>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>17:15</t>
         </is>
       </c>
       <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+22% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Shruti Kulkarni
+27% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="6" t="n"/>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
+      <c r="H7" s="6" t="n"/>
+    </row>
+    <row r="8" ht="52" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
 Siddhartha Kusuma
-20% pred | 20% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>17:15</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-20% pred | 20% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Shruti Kulkarni
-28% pred | 28% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="n"/>
+17% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G8" s="6" t="n"/>
       <c r="H8" s="6" t="n"/>
     </row>
     <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>18:15</t>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>19:45</t>
         </is>
       </c>
       <c r="B9" s="6" t="n"/>
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-17% pred | 17% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
+Kajol Kanchan
+15% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="n"/>
       <c r="H9" s="6" t="n"/>
-    </row>
-    <row r="10" ht="52" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>19:45</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-15% pred | 15% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1039,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1118,8 +1076,8 @@
         <is>
           <t>Copper + Cloves Mat 57
 Shruti Kulkarni
-12% pred | 12% hist
-[PROTECT_EXACT]</t>
+12% pred | 0% hist
+[]</t>
         </is>
       </c>
       <c r="C3" s="6" t="n"/>
@@ -1143,152 +1101,131 @@
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
-17% pred | 17% hist
-[PROTECT_EXACT]</t>
+17% pred | 0% hist
+[]</t>
         </is>
       </c>
       <c r="G4" s="6" t="n"/>
       <c r="H4" s="6" t="n"/>
     </row>
     <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+18% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
 Pushyank Nahar
 20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Pushyank Nahar
-46% pred | 46% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="n"/>
-    </row>
-    <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>09:30</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Pushyank Nahar
-21% pred | 21% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
+[]</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n"/>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+46% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="H6" s="6" t="n"/>
     </row>
     <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>11:30</t>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>17:15</t>
         </is>
       </c>
       <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+22% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Shruti Kulkarni
+27% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="6" t="n"/>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
+      <c r="H7" s="6" t="n"/>
+    </row>
+    <row r="8" ht="52" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
 Siddhartha Kusuma
-20% pred | 20% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>17:15</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-20% pred | 20% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Shruti Kulkarni
-28% pred | 28% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="n"/>
+17% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G8" s="6" t="n"/>
       <c r="H8" s="6" t="n"/>
     </row>
     <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>18:15</t>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>19:45</t>
         </is>
       </c>
       <c r="B9" s="6" t="n"/>
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-17% pred | 17% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
+Kajol Kanchan
+15% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="n"/>
       <c r="H9" s="6" t="n"/>
-    </row>
-    <row r="10" ht="52" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>19:45</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-15% pred | 15% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
chore: update schedule assignments, metrics, and output artifacts based on optimized generator logic
</commit_message>
<xml_diff>
--- a/outputs/schedule_copper_cloves.xlsx
+++ b/outputs/schedule_copper_cloves.xlsx
@@ -47,13 +47,13 @@
       <sz val="9"/>
     </font>
     <font>
-      <color rgb="006B21A8"/>
-      <sz val="9"/>
-    </font>
-    <font>
       <b val="1"/>
       <color rgb="0092400E"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="006B21A8"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="8">
@@ -85,12 +85,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8D5FF"/>
+        <fgColor rgb="00FFFBEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFBEB"/>
+        <fgColor rgb="00E8D5FF"/>
       </patternFill>
     </fill>
   </fills>
@@ -139,10 +139,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -509,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -581,14 +581,14 @@
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>08:15</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
-Shruti Kulkarni
-12% pred | 0% hist
+Pushyank Nahar
+33% pred | 0% hist
 []</t>
         </is>
       </c>
@@ -600,55 +600,13 @@
       <c r="H3" s="6" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>07:30</t>
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>09:00</t>
         </is>
       </c>
       <c r="B4" s="6" t="n"/>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-17% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="n"/>
-      <c r="H4" s="6" t="n"/>
-    </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>08:15</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Pushyank Nahar
-18% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-    </row>
-    <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
 Pushyank Nahar
@@ -656,17 +614,66 @@
 []</t>
         </is>
       </c>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+46% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Pushyank Nahar
+21% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+36% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Shruti Kulkarni
+24% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n"/>
       <c r="D6" s="6" t="n"/>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="n"/>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Pushyank Nahar
-46% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="G6" s="6" t="n"/>
       <c r="H6" s="6" t="n"/>
     </row>
     <row r="7" ht="52" customHeight="1">
@@ -676,11 +683,11 @@
         </is>
       </c>
       <c r="B7" s="6" t="n"/>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
-22% pred | 0% hist
+20% pred | 0% hist
 []</t>
         </is>
       </c>
@@ -689,7 +696,7 @@
         <is>
           <t>Copper + Cloves Mat 57
 Shruti Kulkarni
-27% pred | 0% hist
+28% pred | 0% hist
 []</t>
         </is>
       </c>
@@ -698,46 +705,25 @@
       <c r="H7" s="6" t="n"/>
     </row>
     <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>18:15</t>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>19:45</t>
         </is>
       </c>
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="6" t="n"/>
       <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-17% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+18% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="n"/>
       <c r="G8" s="6" t="n"/>
       <c r="H8" s="6" t="n"/>
-    </row>
-    <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>19:45</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-15% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -753,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -825,14 +811,14 @@
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>08:15</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
-Shruti Kulkarni
-12% pred | 0% hist
+Pushyank Nahar
+33% pred | 0% hist
 []</t>
         </is>
       </c>
@@ -844,55 +830,13 @@
       <c r="H3" s="6" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>07:30</t>
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>09:00</t>
         </is>
       </c>
       <c r="B4" s="6" t="n"/>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-17% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="n"/>
-      <c r="H4" s="6" t="n"/>
-    </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>08:15</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Pushyank Nahar
-18% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-    </row>
-    <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
 Pushyank Nahar
@@ -900,17 +844,66 @@
 []</t>
         </is>
       </c>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+46% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Pushyank Nahar
+21% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+36% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Shruti Kulkarni
+24% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n"/>
       <c r="D6" s="6" t="n"/>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="n"/>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Pushyank Nahar
-46% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="G6" s="6" t="n"/>
       <c r="H6" s="6" t="n"/>
     </row>
     <row r="7" ht="52" customHeight="1">
@@ -920,11 +913,11 @@
         </is>
       </c>
       <c r="B7" s="6" t="n"/>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
-22% pred | 0% hist
+20% pred | 0% hist
 []</t>
         </is>
       </c>
@@ -933,7 +926,7 @@
         <is>
           <t>Copper + Cloves Mat 57
 Shruti Kulkarni
-27% pred | 0% hist
+28% pred | 0% hist
 []</t>
         </is>
       </c>
@@ -942,46 +935,25 @@
       <c r="H7" s="6" t="n"/>
     </row>
     <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>18:15</t>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>19:45</t>
         </is>
       </c>
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="6" t="n"/>
       <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-17% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+18% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="n"/>
       <c r="G8" s="6" t="n"/>
       <c r="H8" s="6" t="n"/>
-    </row>
-    <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>19:45</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-15% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -997,7 +969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1069,14 +1041,14 @@
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>08:15</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
-Shruti Kulkarni
-12% pred | 0% hist
+Pushyank Nahar
+33% pred | 0% hist
 []</t>
         </is>
       </c>
@@ -1088,55 +1060,13 @@
       <c r="H3" s="6" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>07:30</t>
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>09:00</t>
         </is>
       </c>
       <c r="B4" s="6" t="n"/>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-17% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="n"/>
-      <c r="H4" s="6" t="n"/>
-    </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>08:15</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Pushyank Nahar
-18% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-    </row>
-    <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
 Pushyank Nahar
@@ -1144,17 +1074,66 @@
 []</t>
         </is>
       </c>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+46% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Pushyank Nahar
+21% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+36% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Shruti Kulkarni
+24% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n"/>
       <c r="D6" s="6" t="n"/>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="n"/>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Pushyank Nahar
-46% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="G6" s="6" t="n"/>
       <c r="H6" s="6" t="n"/>
     </row>
     <row r="7" ht="52" customHeight="1">
@@ -1164,11 +1143,11 @@
         </is>
       </c>
       <c r="B7" s="6" t="n"/>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
-22% pred | 0% hist
+20% pred | 0% hist
 []</t>
         </is>
       </c>
@@ -1177,7 +1156,7 @@
         <is>
           <t>Copper + Cloves Mat 57
 Shruti Kulkarni
-27% pred | 0% hist
+28% pred | 0% hist
 []</t>
         </is>
       </c>
@@ -1186,46 +1165,25 @@
       <c r="H7" s="6" t="n"/>
     </row>
     <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>18:15</t>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>19:45</t>
         </is>
       </c>
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="6" t="n"/>
       <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-17% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+18% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="n"/>
       <c r="G8" s="6" t="n"/>
       <c r="H8" s="6" t="n"/>
-    </row>
-    <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>19:45</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-15% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
refactor: update scoring weights and regenerate scheduler state, outputs, and web assets
</commit_message>
<xml_diff>
--- a/outputs/schedule_copper_cloves.xlsx
+++ b/outputs/schedule_copper_cloves.xlsx
@@ -47,13 +47,13 @@
       <sz val="9"/>
     </font>
     <font>
+      <color rgb="006B21A8"/>
+      <sz val="9"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="0092400E"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <color rgb="006B21A8"/>
-      <sz val="9"/>
     </font>
   </fonts>
   <fills count="8">
@@ -85,12 +85,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFBEB"/>
+        <fgColor rgb="00E8D5FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8D5FF"/>
+        <fgColor rgb="00FFFBEB"/>
       </patternFill>
     </fill>
   </fills>
@@ -139,10 +139,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -509,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -581,14 +581,14 @@
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>08:15</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
-Pushyank Nahar
-33% pred | 0% hist
+Shruti Kulkarni
+12% pred | 0% hist
 []</t>
         </is>
       </c>
@@ -600,13 +600,55 @@
       <c r="H3" s="6" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+17% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+18% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
 Pushyank Nahar
@@ -614,116 +656,109 @@
 []</t>
         </is>
       </c>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Pushyank Nahar
-46% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="n"/>
-    </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>09:30</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Pushyank Nahar
-21% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-36% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-    </row>
-    <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>10:30</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Shruti Kulkarni
-24% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="n"/>
       <c r="D6" s="6" t="n"/>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+46% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="H6" s="6" t="n"/>
     </row>
     <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>17:15</t>
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>09:30</t>
         </is>
       </c>
       <c r="B7" s="6" t="n"/>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="C7" s="6" t="n"/>
       <c r="D7" s="6" t="n"/>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Shruti Kulkarni
-28% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+22% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G7" s="6" t="n"/>
       <c r="H7" s="6" t="n"/>
     </row>
     <row r="8" ht="52" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="B8" s="6" t="n"/>
-      <c r="C8" s="6" t="n"/>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+23% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="D8" s="6" t="n"/>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-18% pred | 0% hist
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Shruti Kulkarni
+27% pred | 0% hist
 []</t>
         </is>
       </c>
       <c r="F8" s="6" t="n"/>
       <c r="G8" s="6" t="n"/>
       <c r="H8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Siddhartha Kusuma
+17% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="52" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+15% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -739,7 +774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -811,14 +846,14 @@
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>08:15</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
-Pushyank Nahar
-33% pred | 0% hist
+Shruti Kulkarni
+12% pred | 0% hist
 []</t>
         </is>
       </c>
@@ -830,13 +865,55 @@
       <c r="H3" s="6" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+17% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+18% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
 Pushyank Nahar
@@ -844,116 +921,109 @@
 []</t>
         </is>
       </c>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Pushyank Nahar
-46% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="n"/>
-    </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>09:30</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Pushyank Nahar
-21% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-36% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-    </row>
-    <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>10:30</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Shruti Kulkarni
-24% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="n"/>
       <c r="D6" s="6" t="n"/>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+46% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="H6" s="6" t="n"/>
     </row>
     <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>17:15</t>
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>09:30</t>
         </is>
       </c>
       <c r="B7" s="6" t="n"/>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="C7" s="6" t="n"/>
       <c r="D7" s="6" t="n"/>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Shruti Kulkarni
-28% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+22% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G7" s="6" t="n"/>
       <c r="H7" s="6" t="n"/>
     </row>
     <row r="8" ht="52" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="B8" s="6" t="n"/>
-      <c r="C8" s="6" t="n"/>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+23% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="D8" s="6" t="n"/>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-18% pred | 0% hist
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Shruti Kulkarni
+27% pred | 0% hist
 []</t>
         </is>
       </c>
       <c r="F8" s="6" t="n"/>
       <c r="G8" s="6" t="n"/>
       <c r="H8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Siddhartha Kusuma
+17% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="52" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+15% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -969,7 +1039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1041,14 +1111,14 @@
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>08:15</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
-Pushyank Nahar
-33% pred | 0% hist
+Shruti Kulkarni
+12% pred | 0% hist
 []</t>
         </is>
       </c>
@@ -1060,13 +1130,55 @@
       <c r="H3" s="6" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+17% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+18% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
 Pushyank Nahar
@@ -1074,116 +1186,109 @@
 []</t>
         </is>
       </c>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Pushyank Nahar
-46% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="n"/>
-    </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>09:30</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Pushyank Nahar
-21% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-36% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-    </row>
-    <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>10:30</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Shruti Kulkarni
-24% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="n"/>
       <c r="D6" s="6" t="n"/>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+46% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="H6" s="6" t="n"/>
     </row>
     <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>17:15</t>
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>09:30</t>
         </is>
       </c>
       <c r="B7" s="6" t="n"/>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="C7" s="6" t="n"/>
       <c r="D7" s="6" t="n"/>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Shruti Kulkarni
-28% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+22% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G7" s="6" t="n"/>
       <c r="H7" s="6" t="n"/>
     </row>
     <row r="8" ht="52" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="B8" s="6" t="n"/>
-      <c r="C8" s="6" t="n"/>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+23% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="D8" s="6" t="n"/>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-18% pred | 0% hist
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Shruti Kulkarni
+27% pred | 0% hist
 []</t>
         </is>
       </c>
       <c r="F8" s="6" t="n"/>
       <c r="G8" s="6" t="n"/>
       <c r="H8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Siddhartha Kusuma
+17% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="52" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+15% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
update: refresh class metrics, schedules, and pipeline state data while adding local testing scripts
</commit_message>
<xml_diff>
--- a/outputs/schedule_copper_cloves.xlsx
+++ b/outputs/schedule_copper_cloves.xlsx
@@ -693,11 +693,32 @@
     <row r="8" ht="52" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Siddhartha Kusuma
+16% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
           <t>17:15</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
@@ -705,8 +726,8 @@
 []</t>
         </is>
       </c>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
 Shruti Kulkarni
@@ -714,28 +735,7 @@
 []</t>
         </is>
       </c>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="6" t="n"/>
-    </row>
-    <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>18:15</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-17% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="n"/>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -958,11 +958,32 @@
     <row r="8" ht="52" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Siddhartha Kusuma
+16% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
           <t>17:15</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
@@ -970,8 +991,8 @@
 []</t>
         </is>
       </c>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
 Shruti Kulkarni
@@ -979,28 +1000,7 @@
 []</t>
         </is>
       </c>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="6" t="n"/>
-    </row>
-    <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>18:15</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-17% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="n"/>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -1223,11 +1223,32 @@
     <row r="8" ht="52" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Siddhartha Kusuma
+16% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
           <t>17:15</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
@@ -1235,8 +1256,8 @@
 []</t>
         </is>
       </c>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
 Shruti Kulkarni
@@ -1244,28 +1265,7 @@
 []</t>
         </is>
       </c>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="6" t="n"/>
-    </row>
-    <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>18:15</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-17% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="n"/>
       <c r="H9" s="6" t="n"/>
     </row>

</xml_diff>

<commit_message>
Refactor code structure and remove redundant sections for improved readability and maintainability
</commit_message>
<xml_diff>
--- a/outputs/schedule_copper_cloves.xlsx
+++ b/outputs/schedule_copper_cloves.xlsx
@@ -39,11 +39,11 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="0092400E"/>
+      <color rgb="00555577"/>
       <sz val="10"/>
     </font>
     <font>
-      <color rgb="000C4A6E"/>
+      <color rgb="006B21A8"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -61,17 +61,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFBEB"/>
+        <fgColor rgb="00F5F5F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8D5FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FAFAFA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D5F2F8"/>
       </patternFill>
     </fill>
   </fills>
@@ -115,10 +115,10 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -556,23 +556,23 @@
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
 Chaitanya Nahar
-31% pred | 0% hist
+32% pred | 0% hist
 []</t>
         </is>
       </c>
-      <c r="H3" s="5" t="n"/>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -660,23 +660,23 @@
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
 Chaitanya Nahar
-31% pred | 0% hist
+32% pred | 0% hist
 []</t>
         </is>
       </c>
-      <c r="H3" s="5" t="n"/>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -764,23 +764,23 @@
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
 Chaitanya Nahar
-31% pred | 0% hist
+32% pred | 0% hist
 []</t>
         </is>
       </c>
-      <c r="H3" s="5" t="n"/>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Add satellite top-up functionality for Copper & Cloves and Courtside schedules
- Implemented `_satellite_top_up_schedule` function to add classes until target count is reached.
- Updated schedule files to reflect new classes for Copper & Cloves on 2026-05-04 and 2026-05-05.
- Modified scorecard and schedule data to account for new classes and updated metrics.
- Enhanced natural language processing to recognize "populate" as a valid command for schedule modifications.
- Adjusted various JSON and CSV outputs to include new class details and updated statistics.
</commit_message>
<xml_diff>
--- a/outputs/schedule_copper_cloves.xlsx
+++ b/outputs/schedule_copper_cloves.xlsx
@@ -668,7 +668,14 @@
           <t>12:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n"/>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+60% pred | 0% hist
+[MANUAL]</t>
+        </is>
+      </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
@@ -697,7 +704,14 @@
         </is>
       </c>
       <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+60% pred | 0% hist
+[MANUAL]</t>
+        </is>
+      </c>
       <c r="D8" s="5" t="n"/>
       <c r="E8" s="5" t="n"/>
       <c r="F8" s="5" t="n"/>
@@ -919,7 +933,14 @@
           <t>12:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n"/>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+60% pred | 0% hist
+[MANUAL]</t>
+        </is>
+      </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
@@ -948,7 +969,14 @@
         </is>
       </c>
       <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+60% pred | 0% hist
+[MANUAL]</t>
+        </is>
+      </c>
       <c r="D8" s="5" t="n"/>
       <c r="E8" s="5" t="n"/>
       <c r="F8" s="5" t="n"/>
@@ -1170,7 +1198,14 @@
           <t>12:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n"/>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+60% pred | 0% hist
+[MANUAL]</t>
+        </is>
+      </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
@@ -1199,7 +1234,14 @@
         </is>
       </c>
       <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+60% pred | 0% hist
+[MANUAL]</t>
+        </is>
+      </c>
       <c r="D8" s="5" t="n"/>
       <c r="E8" s="5" t="n"/>
       <c r="F8" s="5" t="n"/>

</xml_diff>

<commit_message>
Add schedule data for August 10, 2026
</commit_message>
<xml_diff>
--- a/outputs/schedule_copper_cloves.xlsx
+++ b/outputs/schedule_copper_cloves.xlsx
@@ -47,13 +47,13 @@
       <sz val="9"/>
     </font>
     <font>
-      <color rgb="000C4A6E"/>
-      <sz val="9"/>
-    </font>
-    <font>
       <b val="1"/>
       <color rgb="00555577"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="000C4A6E"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="8">
@@ -85,12 +85,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D5F2F8"/>
+        <fgColor rgb="00F5F5F8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F5F5F8"/>
+        <fgColor rgb="00D5F2F8"/>
       </patternFill>
     </fill>
   </fills>
@@ -139,10 +139,10 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -509,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -525,7 +525,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Copper &amp; Cloves  |  Max Score  |  Week of 2026-05-04</t>
+          <t>Copper &amp; Cloves  |  Max Score  |  Week of 2026-08-10</t>
         </is>
       </c>
     </row>
@@ -538,113 +538,120 @@
       <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Monday
-4-May</t>
+10-Aug</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Tuesday
-5-May</t>
+11-Aug</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Wednesday
-6-May</t>
+12-Aug</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Thursday
-7-May</t>
+13-Aug</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Friday
-8-May</t>
+14-Aug</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Saturday
-9-May</t>
+15-Aug</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Sunday
-10-May</t>
+16-Aug</t>
         </is>
       </c>
     </row>
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="B3" s="5" t="n"/>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
+      <c r="C3" s="5" t="n"/>
       <c r="D3" s="5" t="n"/>
       <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+38% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G3" s="5" t="n"/>
       <c r="H3" s="5" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="n"/>
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Shruti Kulkarni
+24% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="5" t="n"/>
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="5" t="n"/>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Chaitanya Nahar
-31% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="G4" s="5" t="n"/>
       <c r="H4" s="5" t="n"/>
     </row>
     <row r="5" ht="52" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Shruti Kulkarni
+15% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Siddhartha Kusuma
+30% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="5" t="n"/>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-60% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n"/>
     </row>
     <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>12:00</t>
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>11:15</t>
         </is>
       </c>
       <c r="B6" s="5" t="n"/>
@@ -652,113 +659,57 @@
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Siddhartha Kusuma
 60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
+[]</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="n"/>
     </row>
     <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Pushyank Nahar
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="5" t="n"/>
       <c r="D7" s="5" t="n"/>
       <c r="E7" s="5" t="n"/>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
 Chaitanya Nahar
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
+100% pred | 0% hist
+[]</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>19:30</t>
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B8" s="5" t="n"/>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
+      <c r="C8" s="5" t="n"/>
       <c r="D8" s="5" t="n"/>
       <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Siddhartha Kusuma
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G8" s="5" t="n"/>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>20:30</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Pushyank Nahar
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Pushyank Nahar
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
+      <c r="H8" s="5" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -774,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -790,7 +741,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Copper &amp; Cloves  |  Trainer Hours  |  Week of 2026-05-04</t>
+          <t>Copper &amp; Cloves  |  Trainer Hours  |  Week of 2026-08-10</t>
         </is>
       </c>
     </row>
@@ -803,113 +754,120 @@
       <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Monday
-4-May</t>
+10-Aug</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Tuesday
-5-May</t>
+11-Aug</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Wednesday
-6-May</t>
+12-Aug</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Thursday
-7-May</t>
+13-Aug</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Friday
-8-May</t>
+14-Aug</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Saturday
-9-May</t>
+15-Aug</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Sunday
-10-May</t>
+16-Aug</t>
         </is>
       </c>
     </row>
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="B3" s="5" t="n"/>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
+      <c r="C3" s="5" t="n"/>
       <c r="D3" s="5" t="n"/>
       <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+38% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G3" s="5" t="n"/>
       <c r="H3" s="5" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="n"/>
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Shruti Kulkarni
+24% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="5" t="n"/>
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="5" t="n"/>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Chaitanya Nahar
-31% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="G4" s="5" t="n"/>
       <c r="H4" s="5" t="n"/>
     </row>
     <row r="5" ht="52" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Shruti Kulkarni
+15% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Siddhartha Kusuma
+30% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="5" t="n"/>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-60% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n"/>
     </row>
     <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>12:00</t>
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>11:15</t>
         </is>
       </c>
       <c r="B6" s="5" t="n"/>
@@ -917,113 +875,57 @@
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Siddhartha Kusuma
 60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
+[]</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="n"/>
     </row>
     <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Pushyank Nahar
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="5" t="n"/>
       <c r="D7" s="5" t="n"/>
       <c r="E7" s="5" t="n"/>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
 Chaitanya Nahar
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
+100% pred | 0% hist
+[]</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>19:30</t>
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B8" s="5" t="n"/>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
+      <c r="C8" s="5" t="n"/>
       <c r="D8" s="5" t="n"/>
       <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Siddhartha Kusuma
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G8" s="5" t="n"/>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>20:30</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Pushyank Nahar
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Pushyank Nahar
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
+      <c r="H8" s="5" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1039,7 +941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1055,7 +957,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Copper &amp; Cloves  |  Class Variety  |  Week of 2026-05-04</t>
+          <t>Copper &amp; Cloves  |  Class Variety  |  Week of 2026-08-10</t>
         </is>
       </c>
     </row>
@@ -1068,113 +970,120 @@
       <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Monday
-4-May</t>
+10-Aug</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Tuesday
-5-May</t>
+11-Aug</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Wednesday
-6-May</t>
+12-Aug</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Thursday
-7-May</t>
+13-Aug</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Friday
-8-May</t>
+14-Aug</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Saturday
-9-May</t>
+15-Aug</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Sunday
-10-May</t>
+16-Aug</t>
         </is>
       </c>
     </row>
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="B3" s="5" t="n"/>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
+      <c r="C3" s="5" t="n"/>
       <c r="D3" s="5" t="n"/>
       <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+38% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G3" s="5" t="n"/>
       <c r="H3" s="5" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="n"/>
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Shruti Kulkarni
+24% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="5" t="n"/>
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="5" t="n"/>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Chaitanya Nahar
-31% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="G4" s="5" t="n"/>
       <c r="H4" s="5" t="n"/>
     </row>
     <row r="5" ht="52" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Shruti Kulkarni
+15% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Siddhartha Kusuma
+30% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="5" t="n"/>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-60% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n"/>
     </row>
     <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>12:00</t>
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>11:15</t>
         </is>
       </c>
       <c r="B6" s="5" t="n"/>
@@ -1182,113 +1091,57 @@
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Siddhartha Kusuma
 60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
+[]</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="n"/>
     </row>
     <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Pushyank Nahar
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="5" t="n"/>
       <c r="D7" s="5" t="n"/>
       <c r="E7" s="5" t="n"/>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
 Chaitanya Nahar
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
+100% pred | 0% hist
+[]</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>19:30</t>
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B8" s="5" t="n"/>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
+      <c r="C8" s="5" t="n"/>
       <c r="D8" s="5" t="n"/>
       <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Siddhartha Kusuma
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G8" s="5" t="n"/>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>20:30</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Pushyank Nahar
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Pushyank Nahar
-60% pred | 0% hist
-[MANUAL]</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
+      <c r="H8" s="5" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Add schedule validator and validation report generation
- Implemented a new schedule validator in `agents/schedule_validator.py` to ensure compliance with hard rules for scheduling classes.
- The validator checks various conditions such as class timings, trainer qualifications, and location-specific rules.
- Introduced a function to validate a schedule file and update it with any violations found.
- Created a sample validation report in `state/06_validation_report.json` detailing violations and counts by rule.
</commit_message>
<xml_diff>
--- a/outputs/schedule_copper_cloves.xlsx
+++ b/outputs/schedule_copper_cloves.xlsx
@@ -43,10 +43,6 @@
       <sz val="10"/>
     </font>
     <font>
-      <color rgb="000C4A6E"/>
-      <sz val="9"/>
-    </font>
-    <font>
       <color rgb="006B21A8"/>
       <sz val="9"/>
     </font>
@@ -54,6 +50,10 @@
       <b val="1"/>
       <color rgb="00555577"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="000C4A6E"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="8">
@@ -80,17 +80,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D5F2F8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00E8D5FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F5F5F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D5F2F8"/>
       </patternFill>
     </fill>
   </fills>
@@ -139,10 +139,10 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -581,85 +581,64 @@
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="B3" s="5" t="n"/>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Pushyank Nahar
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="C3" s="5" t="n"/>
       <c r="D3" s="5" t="n"/>
       <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+38% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G3" s="5" t="n"/>
       <c r="H3" s="5" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>11:00</t>
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>11:15</t>
         </is>
       </c>
       <c r="B4" s="5" t="n"/>
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="5" t="n"/>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
-Shruti Kulkarni
-35% pred | 0% hist
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Siddhartha Kusuma
+20% pred | 0% hist
 []</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="H4" s="5" t="n"/>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
-25% pred | 0% hist
+23% pred | 0% hist
 []</t>
         </is>
       </c>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-    </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>11:15</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Shruti Kulkarni
-15% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Siddhartha Kusuma
-30% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="D5" s="5" t="n"/>
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="5" t="n"/>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-60% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n"/>
     </row>
   </sheetData>
@@ -748,85 +727,64 @@
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="B3" s="5" t="n"/>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Pushyank Nahar
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="C3" s="5" t="n"/>
       <c r="D3" s="5" t="n"/>
       <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+38% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G3" s="5" t="n"/>
       <c r="H3" s="5" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>11:00</t>
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>11:15</t>
         </is>
       </c>
       <c r="B4" s="5" t="n"/>
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="5" t="n"/>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
-Shruti Kulkarni
-35% pred | 0% hist
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Siddhartha Kusuma
+20% pred | 0% hist
 []</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="H4" s="5" t="n"/>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
-25% pred | 0% hist
+23% pred | 0% hist
 []</t>
         </is>
       </c>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-    </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>11:15</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Shruti Kulkarni
-15% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Siddhartha Kusuma
-30% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="D5" s="5" t="n"/>
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="5" t="n"/>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-60% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n"/>
     </row>
   </sheetData>
@@ -915,85 +873,64 @@
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="B3" s="5" t="n"/>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Pushyank Nahar
-20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="C3" s="5" t="n"/>
       <c r="D3" s="5" t="n"/>
       <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+38% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G3" s="5" t="n"/>
       <c r="H3" s="5" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>11:00</t>
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>11:15</t>
         </is>
       </c>
       <c r="B4" s="5" t="n"/>
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="5" t="n"/>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
-Shruti Kulkarni
-35% pred | 0% hist
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Siddhartha Kusuma
+20% pred | 0% hist
 []</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="H4" s="5" t="n"/>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
-25% pred | 0% hist
+23% pred | 0% hist
 []</t>
         </is>
       </c>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-    </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>11:15</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Shruti Kulkarni
-15% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Siddhartha Kusuma
-30% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="D5" s="5" t="n"/>
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="5" t="n"/>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-60% pred | 0% hist
-[]</t>
-        </is>
-      </c>
+      <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n"/>
     </row>
   </sheetData>

</xml_diff>